<commit_message>
fix(web): persistir alertas invitado manual y alinear Excel piloto
Guarda meta local del drawer tras create; regenera invitados-validacion-manual.xlsx sin preferencia_control. Incluye Playwright E2E, Sentry opcional, npm run dev en raíz y evidencias sesión 2026-06-24.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/pilot/invitados-validacion-manual.xlsx
+++ b/docs/pilot/invitados-validacion-manual.xlsx
@@ -1,21 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_50DB384901DAD9F2697B24A73A44F4AD80B56C0B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC6A472A-3708-4764-9475-BAC196376B7B}"/>
-  <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="invitados" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="invitados" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="instrucciones" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="32">
   <si>
     <t>nombre</t>
   </si>
@@ -44,9 +41,6 @@
     <t>separar_acompanante</t>
   </si>
   <si>
-    <t>preferencia_control</t>
-  </si>
-  <si>
     <t>Ana Garcia Lopez</t>
   </si>
   <si>
@@ -62,15 +56,15 @@
     <t>Familia novia</t>
   </si>
   <si>
+    <t>Intolerancia lactosa</t>
+  </si>
+  <si>
     <t>PAREJA_001</t>
   </si>
   <si>
     <t>false</t>
   </si>
   <si>
-    <t>colaborativo</t>
-  </si>
-  <si>
     <t>Luis Martinez Ruiz</t>
   </si>
   <si>
@@ -105,19 +99,31 @@
   </si>
   <si>
     <t>+34600777888</t>
+  </si>
+  <si>
+    <t>Plantilla de validacion manual piloto Taulamic (4 invitados, 2 parejas).</t>
+  </si>
+  <si>
+    <t>Columnas alineadas con la plantilla descargable desde la UI (sin preferencia_control).</t>
+  </si>
+  <si>
+    <t>Modo colaborativo / anfitrion exclusivo: pantalla Preferencias del evento.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
     </font>
   </fonts>
   <fills count="2">
@@ -140,8 +146,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -480,184 +487,186 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="15.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" t="s">
-        <v>26</v>
-      </c>
-      <c r="I5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J5" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(guest-import,web): MEJ-02 plantilla Excel y UX invitados v2
- Excel: columnas menu_especial, movilidad_reducida y notas_internas; marcas booleanas; mapper y detailMetaByCorreo en respuesta de importacion.

- Web: meta de import en API/hook; barra de seleccion masiva inline, borrado en lote y acciones de fila solo icono con tooltip.

- Admin: setup nav bar y shell; iconos de accesorios del plano mas pequenos con tooltip.

- Tests e2e/unit, piloto xlsx, especificacion y plan Sprint 05.
</commit_message>
<xml_diff>
--- a/docs/pilot/invitados-validacion-manual.xlsx
+++ b/docs/pilot/invitados-validacion-manual.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="34">
   <si>
     <t>nombre</t>
   </si>
@@ -32,7 +32,13 @@
     <t>categoria_2</t>
   </si>
   <si>
-    <t>observaciones</t>
+    <t>menu_especial</t>
+  </si>
+  <si>
+    <t>movilidad_reducida</t>
+  </si>
+  <si>
+    <t>notas_internas</t>
   </si>
   <si>
     <t>acompanante_key</t>
@@ -56,15 +62,15 @@
     <t>Familia novia</t>
   </si>
   <si>
+    <t>X</t>
+  </si>
+  <si>
     <t>Intolerancia lactosa</t>
   </si>
   <si>
     <t>PAREJA_001</t>
   </si>
   <si>
-    <t>false</t>
-  </si>
-  <si>
     <t>Luis Martinez Ruiz</t>
   </si>
   <si>
@@ -104,7 +110,7 @@
     <t>Plantilla de validacion manual piloto Taulamic (4 invitados, 2 parejas).</t>
   </si>
   <si>
-    <t>Columnas alineadas con la plantilla descargable desde la UI (sin preferencia_control).</t>
+    <t>Marcas: deja vacio (no) o escribe X / Si en menu_especial, movilidad_reducida y separar_acompanante.</t>
   </si>
   <si>
     <t>Modo colaborativo / anfitrion exclusivo: pantalla Preferencias del evento.</t>
@@ -488,10 +494,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -519,121 +525,151 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
         <v>15</v>
       </c>
-      <c r="I2" t="s">
-        <v>16</v>
+      <c r="F3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" t="s">
-        <v>16</v>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" t="s">
+        <v>14</v>
+      </c>
+      <c r="J4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K4" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H4" t="s">
-        <v>25</v>
-      </c>
-      <c r="I4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
         <v>26</v>
       </c>
-      <c r="B5" t="s">
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" t="s">
         <v>27</v>
       </c>
-      <c r="C5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I5" t="s">
-        <v>16</v>
+      <c r="K5" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -652,17 +688,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>